<commit_message>
removed an incorrect folder reference
</commit_message>
<xml_diff>
--- a/scenario_variables/other_experiment_data/dev0/sub0/run0demand_scenarios188.xlsx
+++ b/scenario_variables/other_experiment_data/dev0/sub0/run0demand_scenarios188.xlsx
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>28725.35614758425</v>
+        <v>40190.99045104837</v>
       </c>
     </row>
     <row r="3">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>23963.01774121611</v>
+        <v>26930.440894984</v>
       </c>
     </row>
     <row r="6">
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>14928.8320178776</v>
+        <v>15957.97157980884</v>
       </c>
     </row>
     <row r="9">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>29138.17913844815</v>
+        <v>36983.83342706213</v>
       </c>
     </row>
     <row r="12">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>7284.544784612039</v>
+        <v>9245.958356765534</v>
       </c>
     </row>
     <row r="14">
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>46487.69937914996</v>
+        <v>82861.88528868358</v>
       </c>
     </row>
     <row r="15">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>11621.98641144057</v>
+        <v>8986.736168046045</v>
       </c>
     </row>
     <row r="18">
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>36844.09611630544</v>
+        <v>31648.64364577689</v>
       </c>
     </row>
     <row r="21">
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>30755.76046864681</v>
+        <v>22904.98327809984</v>
       </c>
     </row>
     <row r="24">
@@ -977,7 +977,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>10739.47105274393</v>
+        <v>11615.48162237537</v>
       </c>
     </row>
     <row r="27">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>23255.36026151579</v>
+        <v>21610.49070051643</v>
       </c>
     </row>
     <row r="30">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>5813.840065378947</v>
+        <v>5402.622675129107</v>
       </c>
     </row>
     <row r="32">
@@ -1103,7 +1103,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>43048.73460781306</v>
+        <v>49959.84799307334</v>
       </c>
     </row>
     <row r="33">
@@ -1166,7 +1166,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>10753.51342411154</v>
+        <v>18348.66607439264</v>
       </c>
     </row>
     <row r="36">
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>26814.71703674526</v>
+        <v>29940.06350108088</v>
       </c>
     </row>
     <row r="39">
@@ -1292,7 +1292,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>10650.39816506652</v>
+        <v>24816.43017160125</v>
       </c>
     </row>
     <row r="42">
@@ -1355,7 +1355,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>6031.558128076127</v>
+        <v>13639.0970986297</v>
       </c>
     </row>
     <row r="45">
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>16626.27482455417</v>
+        <v>21127.95378286267</v>
       </c>
     </row>
     <row r="48">
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>4156.568706138542</v>
+        <v>5281.988445715667</v>
       </c>
     </row>
     <row r="50">
@@ -1481,7 +1481,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>34807.53319498364</v>
+        <v>74257.33618135186</v>
       </c>
     </row>
     <row r="51">
@@ -1544,7 +1544,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>13678.42749723228</v>
+        <v>11273.03350810083</v>
       </c>
     </row>
     <row r="54">
@@ -1607,7 +1607,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>18189.81943359092</v>
+        <v>26250.66310764663</v>
       </c>
     </row>
     <row r="57">
@@ -1670,7 +1670,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>14407.72223998532</v>
+        <v>18635.31259928037</v>
       </c>
     </row>
     <row r="60">
@@ -1733,7 +1733,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>17996.18288345583</v>
+        <v>5658.637493669546</v>
       </c>
     </row>
     <row r="63">
@@ -1796,7 +1796,7 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>18645.34219708079</v>
+        <v>23208.531500607</v>
       </c>
     </row>
     <row r="66">
@@ -1838,7 +1838,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>4661.335549270197</v>
+        <v>5802.13287515175</v>
       </c>
     </row>
     <row r="68">
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>51012.92307031886</v>
+        <v>61725.57653981759</v>
       </c>
     </row>
     <row r="69">
@@ -1922,7 +1922,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>7157.194301699537</v>
+        <v>9628.90537728108</v>
       </c>
     </row>
     <row r="72">
@@ -1985,7 +1985,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>20917.12956606113</v>
+        <v>46623.14095432577</v>
       </c>
     </row>
     <row r="75">
@@ -2048,7 +2048,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>25831.91942282399</v>
+        <v>15624.54129082924</v>
       </c>
     </row>
     <row r="78">
@@ -2111,7 +2111,7 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>8183.774084666365</v>
+        <v>12134.74328315236</v>
       </c>
     </row>
     <row r="81">
@@ -2174,7 +2174,7 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>22254.18811007404</v>
+        <v>18132.27797221037</v>
       </c>
     </row>
     <row r="84">
@@ -2216,7 +2216,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>5563.547027518509</v>
+        <v>4533.069493052592</v>
       </c>
     </row>
     <row r="86">
@@ -2237,7 +2237,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>40990.41965121793</v>
+        <v>75105.77135241017</v>
       </c>
     </row>
     <row r="87">
@@ -2300,7 +2300,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>11406.14843827521</v>
+        <v>18430.10214286862</v>
       </c>
     </row>
     <row r="90">
@@ -2363,7 +2363,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>20487.20040827952</v>
+        <v>25060.01133526014</v>
       </c>
     </row>
     <row r="93">
@@ -2426,7 +2426,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>38892.08638381703</v>
+        <v>26757.11741137459</v>
       </c>
     </row>
     <row r="96">
@@ -2489,7 +2489,7 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>12449.38540723275</v>
+        <v>9225.958393803494</v>
       </c>
     </row>
     <row r="99">
@@ -2552,7 +2552,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>13653.7344262646</v>
+        <v>10709.80913479684</v>
       </c>
     </row>
     <row r="102">
@@ -2594,7 +2594,7 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>3413.43360656615</v>
+        <v>2677.45228369921</v>
       </c>
     </row>
     <row r="104">
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>62338.17368154784</v>
+        <v>43241.51092060348</v>
       </c>
     </row>
     <row r="105">
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>7921.836312608667</v>
+        <v>12535.1620439569</v>
       </c>
     </row>
     <row r="108">
@@ -2741,7 +2741,7 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>26566.47696253567</v>
+        <v>34362.00937667093</v>
       </c>
     </row>
     <row r="111">
@@ -2804,7 +2804,7 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>10302.47407090168</v>
+        <v>34081.61403799687</v>
       </c>
     </row>
     <row r="114">
@@ -2867,7 +2867,7 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>7519.302316630885</v>
+        <v>10686.01619204045</v>
       </c>
     </row>
     <row r="117">
@@ -2930,7 +2930,7 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>21181.16741521474</v>
+        <v>17529.74785740435</v>
       </c>
     </row>
     <row r="120">
@@ -2972,7 +2972,7 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>5295.291853803686</v>
+        <v>4382.436964351086</v>
       </c>
     </row>
     <row r="122">
@@ -2993,7 +2993,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>61076.99869993115</v>
+        <v>35202.62139437507</v>
       </c>
     </row>
     <row r="123">
@@ -3056,7 +3056,7 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>13142.63105446239</v>
+        <v>7891.441297004914</v>
       </c>
     </row>
     <row r="126">
@@ -3119,7 +3119,7 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>24132.63788208819</v>
+        <v>14510.80657033599</v>
       </c>
     </row>
     <row r="129">
@@ -3182,7 +3182,7 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>22741.72228308033</v>
+        <v>42455.53706217187</v>
       </c>
     </row>
     <row r="132">
@@ -3245,7 +3245,7 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>6955.542536122148</v>
+        <v>10309.09080551528</v>
       </c>
     </row>
     <row r="135">
@@ -3308,7 +3308,7 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>15680.93474963175</v>
+        <v>16844.80275416341</v>
       </c>
     </row>
     <row r="138">
@@ -3350,7 +3350,7 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>3920.233687407937</v>
+        <v>4211.200688540852</v>
       </c>
     </row>
     <row r="140">
@@ -3371,7 +3371,7 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>43090.41843560319</v>
+        <v>33153.99016446984</v>
       </c>
     </row>
     <row r="141">
@@ -3434,7 +3434,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>16464.20834832093</v>
+        <v>15042.50950331817</v>
       </c>
     </row>
     <row r="144">

</xml_diff>